<commit_message>
Mejoras en el boom
</commit_message>
<xml_diff>
--- a/doc/PRESUPUESTO.xlsx
+++ b/doc/PRESUPUESTO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\diego\Documents\Universidad\S9-MASTER\EMC\MOUNTAIN_IN_THE_POCKET\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDDF55BA-10DA-4E87-80AE-947CE3B3FFD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42319328-43A8-4F36-AAA8-B4E64CFDACC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="34">
   <si>
     <t>PROVEEDOR</t>
   </si>
@@ -107,22 +107,37 @@
     <t>https://es.farnell.com/bourns/3362p-1-103lf/pot-trimmer-10k-3-pin/dp/9354301</t>
   </si>
   <si>
-    <t>CEM-1206S</t>
-  </si>
-  <si>
     <t>Buzzer</t>
   </si>
   <si>
-    <t>https://es.farnell.com/same-sky/cem-1206s/transudct-zumb-mag-92dba-3-8v/dp/4814136</t>
-  </si>
-  <si>
-    <t>Transistor del buzzer</t>
-  </si>
-  <si>
-    <t>Diodo de descarga del buzzer</t>
-  </si>
-  <si>
     <t>LED indicador</t>
+  </si>
+  <si>
+    <t>Pulsador</t>
+  </si>
+  <si>
+    <t>STLED316SMTR</t>
+  </si>
+  <si>
+    <t>Controlador display 7 segmentos</t>
+  </si>
+  <si>
+    <t>https://es.farnell.com/stmicroelectronics/stled316smtr/control-led-keyscan-14-salida/dp/2806851</t>
+  </si>
+  <si>
+    <t>CEM-1205-IC</t>
+  </si>
+  <si>
+    <t>https://es.farnell.com/same-sky/cem-1205-ic/transudct-zumb-mag-92dba-3-6v/dp/4814135#anchorTechnicalDOCS</t>
+  </si>
+  <si>
+    <t>Mosfet del buzzer</t>
+  </si>
+  <si>
+    <t>2N7002</t>
+  </si>
+  <si>
+    <t>https://es.farnell.com/onsemi/2n7002/mosfet-n-ch-60v-115ma-to-263ab/dp/2323152</t>
   </si>
 </sst>
 </file>
@@ -132,7 +147,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -151,6 +166,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -210,11 +233,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -237,8 +261,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Hipervínculo" xfId="2" builtinId="8"/>
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -593,7 +621,7 @@
         <v>7.19</v>
       </c>
       <c r="F3" s="6">
-        <f t="shared" ref="F3:F7" si="0">E3*D3</f>
+        <f t="shared" ref="F3:F9" si="0">E3*D3</f>
         <v>7.19</v>
       </c>
       <c r="G3" s="7" t="s">
@@ -620,7 +648,7 @@
         <f t="shared" si="0"/>
         <v>4.4800000000000004</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -629,23 +657,23 @@
         <v>5</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="D5" s="5">
         <v>1</v>
       </c>
       <c r="E5" s="6">
-        <v>2.23</v>
+        <v>2</v>
       </c>
       <c r="F5" s="6">
-        <f t="shared" si="0"/>
-        <v>2.23</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>19</v>
+        <f>E5*D5</f>
+        <v>2</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.45">
@@ -653,23 +681,23 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D6" s="5">
         <v>1</v>
       </c>
       <c r="E6" s="6">
-        <v>1.1200000000000001</v>
+        <v>2.23</v>
       </c>
       <c r="F6" s="6">
         <f t="shared" si="0"/>
-        <v>1.1200000000000001</v>
+        <v>2.23</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.45">
@@ -677,59 +705,83 @@
         <v>5</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D7" s="5">
         <v>1</v>
       </c>
       <c r="E7" s="6">
-        <v>1.1652</v>
+        <v>1.1200000000000001</v>
       </c>
       <c r="F7" s="6">
         <f t="shared" si="0"/>
-        <v>1.1652</v>
+        <v>1.1200000000000001</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="5" t="s">
         <v>5</v>
       </c>
+      <c r="B8" s="5" t="s">
+        <v>29</v>
+      </c>
       <c r="C8" s="5" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D8" s="5">
         <v>1</v>
       </c>
-      <c r="G8" s="7"/>
+      <c r="E8" s="6">
+        <v>2.17</v>
+      </c>
+      <c r="F8" s="6">
+        <f t="shared" si="0"/>
+        <v>2.17</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="5" t="s">
         <v>5</v>
       </c>
+      <c r="B9" s="5" t="s">
+        <v>32</v>
+      </c>
       <c r="C9" s="5" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D9" s="5">
         <v>1</v>
       </c>
-      <c r="G9" s="7"/>
+      <c r="E9" s="6">
+        <v>2.9</v>
+      </c>
+      <c r="F9" s="6">
+        <f t="shared" si="0"/>
+        <v>2.9</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A10" s="5" t="s">
-        <v>5</v>
-      </c>
       <c r="C10" s="5" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="G10" s="7"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="C11" s="5" t="s">
+        <v>25</v>
+      </c>
       <c r="G11" s="7"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
@@ -778,6 +830,10 @@
       <c r="G26" s="7"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G4" r:id="rId1" xr:uid="{60EF82CD-5EF6-4223-B34F-B18CA6194041}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>